<commit_message>
fixed some formatting issues, removed question regarding dipping into savings
</commit_message>
<xml_diff>
--- a/data/processed/cdf.xlsx
+++ b/data/processed/cdf.xlsx
@@ -1,23 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yipho/anes/cumulative_anes/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5943E686-0FF0-A34C-AA82-FC5CDDA9D98E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4031B544-88F7-3E47-9BBE-07DCD6A14993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="660" windowWidth="14160" windowHeight="15400" xr2:uid="{3E9128F5-EFF8-A641-AEC4-52663B1E9FB6}"/>
-    <workbookView xWindow="14460" yWindow="660" windowWidth="14180" windowHeight="15400" activeTab="1" xr2:uid="{4F174E8A-7303-6243-8ED4-F9DB801B02F5}"/>
+    <workbookView xWindow="14500" yWindow="660" windowWidth="14160" windowHeight="15420" activeTab="1" xr2:uid="{4F174E8A-7303-6243-8ED4-F9DB801B02F5}"/>
   </bookViews>
   <sheets>
     <sheet name="cdf" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -28,7 +40,7 @@
     <author>tc={AB143EFC-31F3-3C45-9383-00A5B85114D7}</author>
   </authors>
   <commentList>
-    <comment ref="B23" authorId="0" shapeId="0" xr:uid="{92CB0C68-B0E4-E84C-8E72-4F12B3D70530}">
+    <comment ref="B22" authorId="0" shapeId="0" xr:uid="{92CB0C68-B0E4-E84C-8E72-4F12B3D70530}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -36,7 +48,7 @@
     2016: Instead of saying near future, 2016 says "next twelve months"</t>
       </text>
     </comment>
-    <comment ref="B29" authorId="1" shapeId="0" xr:uid="{AB143EFC-31F3-3C45-9383-00A5B85114D7}">
+    <comment ref="B28" authorId="1" shapeId="0" xr:uid="{AB143EFC-31F3-3C45-9383-00A5B85114D7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -49,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="881">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1665" uniqueCount="891">
   <si>
     <t>Variable</t>
   </si>
@@ -3880,33 +3892,6 @@
     <t xml:space="preserve">We are interested in how people are getting along financially thesedays. Would you say that [you / you and your family living here] are much better off financially, somewhat better off, about the same, somewhat worse off, or much worse off than you were a year ago? </t>
   </si>
   <si>
-    <t>PRE: HAS R DONE ANY OF THE FOLLOWING - DIPPED INTO SAVINGS</t>
-  </si>
-  <si>
-    <t>2024: V241568d
-1992: V923436
-1984: V840161</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(2024)   
-0. Not mentioned
-1. Mentioned 
-(1992/1984)  
-1.  YES                                                     
-5.  NO  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">(2024)
--9. Refused
--5. Break oﬀ, suﬃcient partial
--1. Inapplicable
-(1992/1984)
-8. DK 
-9. NA
-0. Inap
-</t>
-  </si>
-  <si>
     <t>POST: CSES: STATE OF ECONOMY BETTER OR WORSE OVER PAST 12 MONTHS</t>
   </si>
   <si>
@@ -3916,11 +3901,6 @@
   <si>
     <t>Now for questions on different topics. Do the health benefits of vaccinations generally outweigh the risks, do the risks outweigh the benefits, or is there no difference?
 Are the [health benefits/risks] of vaccinations much greater, moderately greater, or slightly greater?</t>
-  </si>
-  <si>
-    <t>In the past year, have you done any of the following? Mark all that
-apply. (2024)
-IN THE PAST YEAR HAVE YOU (AND YOUR FAMILY) HAD TO USE YOUR SAVINGS TO MAKE ENDS MEET? (1984/1992)</t>
   </si>
   <si>
     <t>When it comes to people trying to improve their financial well- being, do you think it is now easier, harder, or the same as it was 20 years ago?
@@ -3958,6 +3938,89 @@
 5. Oppose a little
 6. Oppose a moderate
 7. Oppose a great deal</t>
+  </si>
+  <si>
+    <t>2024: V241262
+2020: V201301
+2008: V083141a</t>
+  </si>
+  <si>
+    <t>2024: V241265
+2020: V201304
+2008: V083142a</t>
+  </si>
+  <si>
+    <t>2024: V241271
+2020: V201310
+2008: V083144a</t>
+  </si>
+  <si>
+    <t>2024: V241274
+2020: V201313
+2008: V083145a</t>
+  </si>
+  <si>
+    <t>2024: V241268
+2020: V201307
+2008: V083149a</t>
+  </si>
+  <si>
+    <t>2024: V241277
+2020: V201316
+2008: V083140a</t>
+  </si>
+  <si>
+    <t>2024: V241283
+2020: V201322
+2008: V083151a</t>
+  </si>
+  <si>
+    <t>2024: V241280
+2020: V201319
+2008: V083148a</t>
+  </si>
+  <si>
+    <t>(2020/2024)
+1. A lot
+2. A little
+(2008)
+1. A great deal
+2. A moderate amount
+3. A little</t>
+  </si>
+  <si>
+    <t>2024: V241336
+2020: V201379
+2016: V161171</t>
+  </si>
+  <si>
+    <t>POST: CSES: AGREE/DISAGREE: R UNDERSTANDS MOST IMPORTANT POLITICAL ISSUES</t>
+  </si>
+  <si>
+    <t>(2016/2020)
+1. Never
+2. Once in a while
+3. About half the time
+4. Most of the time
+5. All the time
+(2024)
+1. Yes
+2. No</t>
+  </si>
+  <si>
+    <t>How much do you feel it is justified for people to use violence to pursue their political goals in this country?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(2020/2024)
+-9. Refused
+-8. Don’t know
+-1. Inapplicable
+(1968)
+8.  DK                                                   
+9.  NA; NO POST-ELECTION INTERVIEW </t>
+  </si>
+  <si>
+    <t xml:space="preserve">How much do you care who wins the presidential election this fall? </t>
   </si>
 </sst>
 </file>
@@ -4448,7 +4511,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4456,6 +4519,13 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="7" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4837,10 +4907,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B23" dT="2025-11-13T20:41:49.60" personId="{9254EDE6-B7E7-F040-A3D9-36F90150B96F}" id="{92CB0C68-B0E4-E84C-8E72-4F12B3D70530}">
+  <threadedComment ref="B22" dT="2025-11-13T20:41:49.60" personId="{9254EDE6-B7E7-F040-A3D9-36F90150B96F}" id="{92CB0C68-B0E4-E84C-8E72-4F12B3D70530}">
     <text>2016: Instead of saying near future, 2016 says "next twelve months"</text>
   </threadedComment>
-  <threadedComment ref="B29" dT="2025-11-13T22:43:53.76" personId="{9254EDE6-B7E7-F040-A3D9-36F90150B96F}" id="{AB143EFC-31F3-3C45-9383-00A5B85114D7}">
+  <threadedComment ref="B28" dT="2025-11-13T22:43:53.76" personId="{9254EDE6-B7E7-F040-A3D9-36F90150B96F}" id="{AB143EFC-31F3-3C45-9383-00A5B85114D7}">
     <text>All years regard the "transgender policy" to the policy of transgender people using bathrooms related to their gender identity. Does the question summary require the whole concept? or can we just say "Transgender policy"?</text>
   </threadedComment>
 </ThreadedComments>
@@ -6387,7 +6457,7 @@
         <v>71</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>880</v>
+        <v>875</v>
       </c>
       <c r="O32" s="1" t="s">
         <v>313</v>
@@ -8927,14 +8997,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F06C183-D354-5B46-AC5B-69BA44B64C6F}">
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F84"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="21.5" customWidth="1"/>
     <col min="3" max="3" width="20.6640625" customWidth="1"/>
     <col min="4" max="4" width="21.5" customWidth="1"/>
     <col min="5" max="5" width="21.6640625" customWidth="1"/>
-    <col min="6" max="6" width="23.1640625" customWidth="1"/>
+    <col min="6" max="6" width="32.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -8959,7 +9029,7 @@
     </row>
     <row r="2" spans="1:6" ht="147" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>20</v>
@@ -8978,8 +9048,8 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="136" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>31</v>
+      <c r="A3" s="1" t="s">
+        <v>38</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>32</v>
@@ -8998,8 +9068,8 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="136" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>38</v>
+      <c r="A4" s="1" t="s">
+        <v>45</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>39</v>
@@ -9018,8 +9088,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="136" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>45</v>
+      <c r="A5" s="1" t="s">
+        <v>52</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>46</v>
@@ -9039,7 +9109,7 @@
     </row>
     <row r="6" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>53</v>
@@ -9059,13 +9129,13 @@
     </row>
     <row r="7" spans="1:6" ht="306" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>65</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>871</v>
+        <v>867</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>71</v>
@@ -9079,13 +9149,13 @@
     </row>
     <row r="8" spans="1:6" ht="306" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>78</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>872</v>
+        <v>868</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>87</v>
@@ -9099,7 +9169,7 @@
     </row>
     <row r="9" spans="1:6" ht="323" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>91</v>
@@ -9119,7 +9189,7 @@
     </row>
     <row r="10" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="B10" t="s">
         <v>862</v>
@@ -9139,7 +9209,7 @@
     </row>
     <row r="11" spans="1:6" ht="289" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>117</v>
@@ -9159,7 +9229,7 @@
     </row>
     <row r="12" spans="1:6" ht="174" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>130</v>
@@ -9179,7 +9249,7 @@
     </row>
     <row r="13" spans="1:6" ht="202" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>138</v>
@@ -9199,7 +9269,7 @@
     </row>
     <row r="14" spans="1:6" ht="170" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>150</v>
@@ -9217,235 +9287,235 @@
         <v>157</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="170" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" ht="136" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="B15" t="s">
+        <v>159</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>866</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>873</v>
+        <v>168</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>868</v>
+        <v>169</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>869</v>
+        <v>60</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>867</v>
+        <v>172</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="227" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>870</v>
+        <v>174</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>60</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="136" x14ac:dyDescent="0.2">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="306" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>178</v>
+        <v>869</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="223" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>874</v>
+        <v>198</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>189</v>
+        <v>110</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="306" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>870</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="136" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="170" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="306" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>875</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>74</v>
-      </c>
       <c r="F20" s="1" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="170" x14ac:dyDescent="0.2">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="85" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>227</v>
+        <v>237</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>239</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>60</v>
+        <v>146</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="85" x14ac:dyDescent="0.2">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>239</v>
+        <v>245</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>249</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>146</v>
+        <v>27</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="126" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>245</v>
+        <v>256</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>27</v>
+        <v>260</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="102" x14ac:dyDescent="0.2">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="136" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>256</v>
+        <v>265</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>267</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>260</v>
+        <v>227</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>60</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="136" x14ac:dyDescent="0.2">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="170" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>267</v>
+        <v>275</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>871</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>60</v>
+        <v>281</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>282</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="170" x14ac:dyDescent="0.2">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>273</v>
+        <v>286</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>876</v>
+        <v>291</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>281</v>
@@ -9454,421 +9524,762 @@
         <v>282</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="153" x14ac:dyDescent="0.2">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="68" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>281</v>
+        <v>872</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>282</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="238" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>299</v>
+        <v>873</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>877</v>
+        <v>71</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>282</v>
+        <v>314</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="238" x14ac:dyDescent="0.2">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="289" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>303</v>
+        <v>317</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>304</v>
+        <v>318</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>878</v>
+        <v>322</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>71</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>314</v>
+        <v>325</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="289" x14ac:dyDescent="0.2">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="272" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>317</v>
+        <v>328</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>318</v>
+        <v>329</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>322</v>
+        <v>333</v>
       </c>
       <c r="D30" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="153" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>874</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="272" x14ac:dyDescent="0.2">
-      <c r="A31" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>329</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>333</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>335</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>313</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="153" x14ac:dyDescent="0.2">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="204" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>339</v>
+        <v>349</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>879</v>
+        <v>354</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>71</v>
+        <v>356</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="204" x14ac:dyDescent="0.2">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>349</v>
+        <v>360</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>350</v>
+        <v>361</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>354</v>
+        <v>363</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>356</v>
+        <v>884</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>325</v>
+        <v>146</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>363</v>
+        <v>375</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>368</v>
+        <v>884</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>146</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>884</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>146</v>
+      </c>
       <c r="F35" s="1" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>884</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>146</v>
+      </c>
       <c r="F36" s="1" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>884</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>146</v>
+      </c>
       <c r="F37" s="1" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>884</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>146</v>
+      </c>
       <c r="F38" s="1" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>884</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>146</v>
+      </c>
       <c r="F39" s="1" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>884</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>146</v>
+      </c>
       <c r="F40" s="1" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="204" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>282</v>
+      </c>
       <c r="F41" s="1" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="102" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>147</v>
+      </c>
       <c r="F42" s="1" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="136" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>886</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="F43" s="1" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="153" x14ac:dyDescent="0.2">
+      <c r="A44" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>887</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="F44" s="1" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="85" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>888</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>282</v>
+      </c>
       <c r="F45" s="1" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="221" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>889</v>
+      </c>
       <c r="F46" s="1" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="85" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>890</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>146</v>
+      </c>
       <c r="F47" s="1" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="102" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>489</v>
+      </c>
       <c r="F48" s="1" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="49" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="136" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>497</v>
+      </c>
       <c r="F49" s="1" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="50" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="170" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>489</v>
+      </c>
       <c r="F50" s="1" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="51" spans="6:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="F51" s="1" t="s">
         <v>504</v>
       </c>
     </row>
-    <row r="52" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A51" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="B51" s="5"/>
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="4" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A52" s="1" t="s">
+        <v>515</v>
+      </c>
       <c r="F52" s="1" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="53" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A53" s="1" t="s">
+        <v>522</v>
+      </c>
       <c r="F53" s="1" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="54" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
+        <v>534</v>
+      </c>
       <c r="F54" s="1" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="55" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
+        <v>546</v>
+      </c>
       <c r="F55" s="1" t="s">
-        <v>545</v>
-      </c>
-    </row>
-    <row r="56" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
+        <v>553</v>
+      </c>
       <c r="F56" s="1" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="57" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A57" s="1" t="s">
+        <v>561</v>
+      </c>
       <c r="F57" s="1" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="58" spans="6:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="F58" s="1" t="s">
         <v>568</v>
       </c>
     </row>
-    <row r="59" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F59" t="s">
+    <row r="58" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A58" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="F58" t="s">
         <v>575</v>
       </c>
     </row>
-    <row r="60" spans="6:6" ht="85" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A59" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A60" s="1" t="s">
+        <v>591</v>
+      </c>
       <c r="F60" s="1" t="s">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="61" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A61" s="1" t="s">
+        <v>604</v>
+      </c>
       <c r="F61" s="1" t="s">
-        <v>603</v>
-      </c>
-    </row>
-    <row r="62" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A62" s="1" t="s">
+        <v>617</v>
+      </c>
       <c r="F62" s="1" t="s">
-        <v>616</v>
-      </c>
-    </row>
-    <row r="63" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
+        <v>628</v>
+      </c>
       <c r="F63" s="1" t="s">
-        <v>627</v>
-      </c>
-    </row>
-    <row r="64" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A64" s="1" t="s">
+        <v>637</v>
+      </c>
       <c r="F64" s="1" t="s">
-        <v>636</v>
-      </c>
-    </row>
-    <row r="65" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
+        <v>648</v>
+      </c>
       <c r="F65" s="1" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="66" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
+        <v>658</v>
+      </c>
       <c r="F66" s="1" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="67" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
+        <v>668</v>
+      </c>
       <c r="F67" s="1" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="68" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
+        <v>677</v>
+      </c>
       <c r="F68" s="1" t="s">
-        <v>676</v>
-      </c>
-    </row>
-    <row r="69" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
+        <v>684</v>
+      </c>
       <c r="F69" s="1" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="70" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+      <c r="A70" s="1" t="s">
+        <v>694</v>
+      </c>
       <c r="F70" s="1" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="71" spans="6:6" ht="68" x14ac:dyDescent="0.2">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
+        <v>708</v>
+      </c>
       <c r="F71" s="1" t="s">
-        <v>707</v>
-      </c>
-    </row>
-    <row r="72" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
+        <v>719</v>
+      </c>
       <c r="F72" s="1" t="s">
-        <v>718</v>
-      </c>
-    </row>
-    <row r="73" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
+        <v>731</v>
+      </c>
       <c r="F73" s="1" t="s">
-        <v>730</v>
-      </c>
-    </row>
-    <row r="74" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
+        <v>741</v>
+      </c>
       <c r="F74" s="1" t="s">
-        <v>740</v>
-      </c>
-    </row>
-    <row r="75" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
+        <v>751</v>
+      </c>
       <c r="F75" s="1" t="s">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="76" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>762</v>
+      </c>
       <c r="F76" s="1" t="s">
-        <v>761</v>
-      </c>
-    </row>
-    <row r="77" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>773</v>
+      </c>
       <c r="F77" s="1" t="s">
-        <v>772</v>
-      </c>
-    </row>
-    <row r="78" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
+        <v>781</v>
+      </c>
       <c r="F78" s="1" t="s">
-        <v>780</v>
-      </c>
-    </row>
-    <row r="79" spans="6:6" ht="68" x14ac:dyDescent="0.2">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
+        <v>793</v>
+      </c>
       <c r="F79" s="1" t="s">
-        <v>792</v>
-      </c>
-    </row>
-    <row r="80" spans="6:6" ht="68" x14ac:dyDescent="0.2">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
+        <v>802</v>
+      </c>
       <c r="F80" s="1" t="s">
-        <v>801</v>
-      </c>
-    </row>
-    <row r="81" spans="6:6" ht="68" x14ac:dyDescent="0.2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
+        <v>811</v>
+      </c>
       <c r="F81" s="1" t="s">
-        <v>810</v>
-      </c>
-    </row>
-    <row r="82" spans="6:6" ht="68" x14ac:dyDescent="0.2">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+      <c r="A82" s="1" t="s">
+        <v>821</v>
+      </c>
       <c r="F82" s="1" t="s">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="83" spans="6:6" ht="68" x14ac:dyDescent="0.2">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
+        <v>831</v>
+      </c>
       <c r="F83" s="1" t="s">
-        <v>830</v>
-      </c>
-    </row>
-    <row r="84" spans="6:6" ht="51" x14ac:dyDescent="0.2">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="A84" s="1" t="s">
+        <v>840</v>
+      </c>
       <c r="F84" s="1" t="s">
-        <v>839</v>
-      </c>
-    </row>
-    <row r="85" spans="6:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="F85" s="1" t="s">
         <v>856</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed some wrong variables, took some variables out, finishing up the cdf
</commit_message>
<xml_diff>
--- a/data/processed/cdf.xlsx
+++ b/data/processed/cdf.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yipho/anes/cumulative_anes/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4031B544-88F7-3E47-9BBE-07DCD6A14993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEFACD6-12C0-D64C-A29F-C380C0E146C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14500" yWindow="660" windowWidth="14160" windowHeight="15420" activeTab="1" xr2:uid="{4F174E8A-7303-6243-8ED4-F9DB801B02F5}"/>
+    <workbookView xWindow="14480" yWindow="660" windowWidth="14160" windowHeight="15400" activeTab="1" xr2:uid="{4F174E8A-7303-6243-8ED4-F9DB801B02F5}"/>
   </bookViews>
   <sheets>
     <sheet name="cdf" sheetId="1" r:id="rId1"/>
@@ -38,6 +38,8 @@
   <authors>
     <author>tc={92CB0C68-B0E4-E84C-8E72-4F12B3D70530}</author>
     <author>tc={AB143EFC-31F3-3C45-9383-00A5B85114D7}</author>
+    <author>tc={DFD8C8CE-6327-EB4D-BAE5-C4F37EA7D163}</author>
+    <author>tc={A687251A-029A-8848-BF21-9CE631347539}</author>
   </authors>
   <commentList>
     <comment ref="B22" authorId="0" shapeId="0" xr:uid="{92CB0C68-B0E4-E84C-8E72-4F12B3D70530}">
@@ -56,12 +58,28 @@
     All years regard the "transgender policy" to the policy of transgender people using bathrooms related to their gender identity. Does the question summary require the whole concept? or can we just say "Transgender policy"?</t>
       </text>
     </comment>
+    <comment ref="A51" authorId="2" shapeId="0" xr:uid="{DFD8C8CE-6327-EB4D-BAE5-C4F37EA7D163}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    For 2024, it just mentions "congress and president" but in the other years 2020/2016, it specifies US senate or House of Reps. </t>
+      </text>
+    </comment>
+    <comment ref="A71" authorId="3" shapeId="0" xr:uid="{A687251A-029A-8848-BF21-9CE631347539}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    in 2016, this is a pre and post question.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1665" uniqueCount="891">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="908">
   <si>
     <t>Variable</t>
   </si>
@@ -4022,12 +4040,259 @@
   <si>
     <t xml:space="preserve">How much do you care who wins the presidential election this fall? </t>
   </si>
+  <si>
+    <t>POST: CSES: HOW INTERESTED IN POLITICS IS R</t>
+  </si>
+  <si>
+    <t>POST: CSES: HOW CLOSELY DOES R FOLLOW POLITICS IN MEDIA</t>
+  </si>
+  <si>
+    <t>How much does Congress pass laws to benefit organizations that spend money to support candidates</t>
+  </si>
+  <si>
+    <t>0. Not mentioned
+1. Mentioned</t>
+  </si>
+  <si>
+    <t>-9. Refused
+-1. Inapplicable
+-8. Don’t know (FTF only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How easy was it for you to get access to a computer with an internet connection to take this survey? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">-9. Refused
+-7. No post-election data, deleted due to incomplete interview
+-6. No post-election interview
+-5. Interview breakoff (sufficient partial IW)
+-4. Technical error
+-1. Inapplicable
+</t>
+  </si>
+  <si>
+    <t>-9. Refused
+-7. No post-election data, deleted due to incomplete interview
+-6. No post-election interview
+-5. Interview breakoff (sufficient partial IW)
+-4. Technical error
+-1. Inapplicable</t>
+  </si>
+  <si>
+    <t>(2024) 
+How important is it for immigrants to adapt to the customs and traditions of the United States?
+(2020/2016)
+Now thinking about minorities in the United States. Do you agree strongly, agree somewhat, neither agree nor disagree, disagree somewhat, or disagree strongly with the following statement? ‘Minorities should adapt to the customs and traditions of the United States.’</t>
+  </si>
+  <si>
+    <t>(2024)
+1. Not at all important
+2. A little important
+3. Moderately important
+4. Very important
+5. Extremely important
+(2020/2016) 
+1. Agree strongly
+2. Agree somewhat
+3. Neither agree nor disagree
+4. Disagree somewhat
+5. Disagree strongly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(2024)
+Are immigrants generally good or bad for America’s economy? 
+(2020/2016)
+And now thinking specifically about immigrants. Do you agree strongly, agree somewhat, neither agree nor disagree, disagree somewhat, or disagree strongly with the following statement? ‘Immigrants are generally good for America’s economy.’
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(2024)
+1. Extremely good
+2. Moderately good
+3. Slightly good
+4. Neither good nor bad
+5. Slightly bad
+6. Moderately bad
+7. Extremely bad
+(2020/2016)
+1. Agree strongly
+2. Agree somewhat
+3. Neither agree nor disagree
+4. Disagree somewhat
+5. Disagree strongly
+</t>
+  </si>
+  <si>
+    <t>POST: CSES: OUT-GROUP ATTITUDES: IMMIGRANTS INCREASE CRIME</t>
+  </si>
+  <si>
+    <t>How much does R agree or disagree that immigrants increase crime rates in the United States?</t>
+  </si>
+  <si>
+    <t>-9. Refused
+-1. Inapplicable
+-6. No post-election interview
+-7. No post data, deleted due</t>
+  </si>
+  <si>
+    <t>010. Protestant, NFS, other, unknown, inter-, or non-denominational
+099. Christian, NFS, unknown, inter-, or non-denominational
+100. 7th Day Adventist
+101. Sabbatarian
+109. Adventist (NFS)
+110. Episcopalian; Anglican
+120. American Baptist Association
+121. American Baptist Churches USA (wrongly aka 'Northern Baptist')
+122. Baptist Bible Fellowship
+123. Baptist General Conference
+124. Missionary Baptist; Baptist Missionary Association of America
+125. Conservative Baptist Association of America
+126. General Association of Regular Baptist Churches; GARB
+127. National Association of Free Will Baptists; United Free Will Baptist
+Church
+128. Primitive Baptist
+129. National Baptist Convention in the USA
+130. National Baptist Convention of America
+131. National Primitive Baptist Convention of the USA
+132. Progressive National Baptist Convention
+133. National Baptist Convention NFS
+134. Reformed Baptist (Calvinist)
+135. Southern Baptist Convention
+136. Full Gospel Baptist Church Fellowship
+149. Baptist (NFS or other Baptist group not in codes 120-135)
+150. United Church of Christ; UCC; Congregational; Congregationalist;
+Evangelical and Reformed Church
+155. Congregational Christian
+160. Church of the Brethren
+161. Brethren (NFS)
+162. Mennonite Church
+163. Moravian Church
+164. Old Order Amish
+165. Quakers; Friends
+166. Evangelical Covenant Church (not Anabaptist in tradition)
+167. Evangelical Free Church, EFC, or EFCA (not Anabaptist in tradition)
+168. Brethren in Christ
+169. Apostolic Christian Church of America
+170. Mennonite Brethren
+171. Apostolic Christian Church Nazarene
+180. Christian and Missionary Alliance; CMA; Alliance
+181. Church of God (Anderson, IN)
+182. Church of the Nazarene
+183. Free Methodist Church
+184. Salvation Army
+185. Wesleyan Church
+186. Church of God of Findlay, OH
+199. Pentecostal (NFS); Church of God (NFS); Holiness (NFS); not ascertained
+whether R Pentecostal or Charismatic (Holin
+200. Plymouth Brethren
+201. Independent Fundamental Churches of America; IFCA
+219. Independent-Fundamentalist (NFS)
+220. Evangelical Lutheran Church in America (formerly Lutheran Church in
+America and The American Lutheran Church); ELCA
+221. Lutheran Church, Missouri Synod; LC-MS
+222. Wisconsin Evangelical Lutheran Synod; WELS
+224. Lutheran Free Church, Association of Free Lutheran Churches, AFLC
+225. Church of the Lutheran Brethren
+229. Lutheran (other or NFS)
+230. United Methodist Church; Evangelical United Brethren
+231. African Methodist Episcopal Church; AME
+232. African Methodist Episcopal Zion Church
+233. Christian Methodist Episcopal Church
+234. Primitive Methodist
+235. Congregational Methodist (fundamentalist)
+240. Fire-Baptized Holiness
+242. Assemblies of the Lord Jesus Christ; AJLC
+243. Church of Our Lord Jesus Christ of the Apostolic Faith; COOLJC
+244. Church of the Lord Jesus Christ of the Apostolic Faith; CLJC
+245. Bible Way Church of Our Lord Jesus Christ
+246. International Bible Way Church of Our Lord Jesus Christ
+249. Methodist (other or NFS)
+250. Assemblies of God; Assembly of God
+251. Church of God (Cleveland, TN)
+252. Church of God (Huntsville, AL)
+253. International Church of the Four Square Gospel
+254. Pentecostal Church of God
+255. Pentecostal Holiness Church
+256. United Pentecostal Church International
+257. Church of God in Christ (incl. not ascertained whether 258)
+258. Church of God in Christ International
+260. Church of God of the Apostolic Faith
+261. Church of God of Prophecy
+262. Vineyard Fellowship
+263. Open Bible Standard Churches
+264. Full Gospel
+267. Apostolic Pentecostal
+270. Presbyterian Church in the U.S.A.
+271. Cumberland Presbyterian Church
+272. Presbyterian Church in America; PCA
+275. Evangelical Presbyterian
+276. Reformed Presbyterian
+279. Presbyterian (other or NFS)
+280. Christian Reformed Church (inaccurately known as 'Dutch Reformed')
+281. Reformed Church in America
+289. Reformed (other or NFS)
+290. Christian Church; Disciples of Christ
+291. Christian Churches and Churches of Christ
+292. Churches of Christ; Church of Christ (NFS)
+293. Christian Congregation
+300. Christian Scientists
+301. Mormons; Latter Day Saints; Community of Christ
+303. Unitarian; Universalist
+304. Jehovah's Witnesses
+305. Unity; Unity Church; Christ Church Unity
+306. Fundamentalist Adventist; Worldwide Church of God; United Church of God
+400. Roman Catholic
+501. Orthodox
+502. Conservative
+503. Reform
+524. Jewish, other, no preference, or NFS
+600. Catholic and  Protestant
+650. Messianic Judaism; Jews for Jesus
+695. More than 1 major religion (e.g., Christian, Jewish, Muslim, etc.)
+700. Greek Rite Catholic
+701. Greek Orthodox
+702. Russian Orthodox
+703. Rumanian Orthodox
+704. Serbian Orthodox
+705. Syrian Orthodox
+706. Armenian Orthodox
+707. Georgian Orthodox
+708. Ukrainian Orthodox
+719. Eastern Orthodox (NFS or other specific Orthodox church)
+720. Muslim; Islam
+721. Buddhist
+722. Hindu
+723. Baha'i; Bahai
+724. American Indian religions; Native American religions
+725. New Age
+726. Wicca; Wiccan
+727. Pagan
+730. Sikh
+732. Konko Church
+735. Spiritualists (not 'spiritual; must refer specifically to
+'Spiritualism' or 'Spiritualists')
+736. Religious Science; Science of Mind (not Scientology; not Christian
+Scientists); Centers for Spiritual Living
+740. Other non-Christian /non-Jewish
+750. Scientology
+790. Religious /ethical cults
+870. Other tradition not codeable to 010-790
+879. R indicates having an affiliation but does not specify one
+880. None
+888. DK whether considers self as part of a particular religion
+889. RF to say if considers self as part of a particular religion</t>
+  </si>
+  <si>
+    <t>2024: V242338
+2020: V202353
+2016: V161307a; V162133</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -4168,6 +4433,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -4511,7 +4782,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4525,7 +4796,12 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="8" xfId="15" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4913,6 +5189,12 @@
   <threadedComment ref="B28" dT="2025-11-13T22:43:53.76" personId="{9254EDE6-B7E7-F040-A3D9-36F90150B96F}" id="{AB143EFC-31F3-3C45-9383-00A5B85114D7}">
     <text>All years regard the "transgender policy" to the policy of transgender people using bathrooms related to their gender identity. Does the question summary require the whole concept? or can we just say "Transgender policy"?</text>
   </threadedComment>
+  <threadedComment ref="A51" dT="2025-11-19T20:35:46.74" personId="{9254EDE6-B7E7-F040-A3D9-36F90150B96F}" id="{DFD8C8CE-6327-EB4D-BAE5-C4F37EA7D163}">
+    <text xml:space="preserve">For 2024, it just mentions "congress and president" but in the other years 2020/2016, it specifies US senate or House of Reps. </text>
+  </threadedComment>
+  <threadedComment ref="A71" dT="2025-11-19T22:17:01.88" personId="{9254EDE6-B7E7-F040-A3D9-36F90150B96F}" id="{A687251A-029A-8848-BF21-9CE631347539}">
+    <text>in 2016, this is a pre and post question.</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
@@ -9000,11 +9282,11 @@
   <dimension ref="A1:F84"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="21.5" customWidth="1"/>
+    <col min="2" max="2" width="79.6640625" customWidth="1"/>
     <col min="3" max="3" width="20.6640625" customWidth="1"/>
     <col min="4" max="4" width="21.5" customWidth="1"/>
     <col min="5" max="5" width="21.6640625" customWidth="1"/>
-    <col min="6" max="6" width="32.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -9023,7 +9305,7 @@
       <c r="E1" s="1" t="s">
         <v>860</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -9407,7 +9689,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="85" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>232</v>
       </c>
@@ -9527,7 +9809,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>294</v>
       </c>
@@ -9887,7 +10169,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="85" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>453</v>
       </c>
@@ -9907,7 +10189,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="221" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>463</v>
       </c>
@@ -9927,7 +10209,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="85" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>471</v>
       </c>
@@ -10007,176 +10289,421 @@
         <v>504</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>505</v>
       </c>
-      <c r="B51" s="5"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
+      <c r="B51" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>513</v>
+      </c>
       <c r="F51" s="4" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="A52" s="1" t="s">
+    <row r="52" spans="1:6" ht="136" x14ac:dyDescent="0.2">
+      <c r="A52" s="4" t="s">
         <v>515</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>62</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>522</v>
       </c>
+      <c r="B53" s="1" t="s">
+        <v>891</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>61</v>
+      </c>
       <c r="F53" s="1" t="s">
         <v>533</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="A54" s="1" t="s">
+    <row r="54" spans="1:6" ht="102" x14ac:dyDescent="0.2">
+      <c r="A54" s="4" t="s">
         <v>534</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>892</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>543</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>545</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>546</v>
       </c>
+      <c r="B55" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>61</v>
+      </c>
       <c r="F55" s="1" t="s">
         <v>552</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>553</v>
       </c>
+      <c r="B56" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>893</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>61</v>
+      </c>
       <c r="F56" s="1" t="s">
         <v>560</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" ht="170" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>561</v>
       </c>
+      <c r="B57" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>61</v>
+      </c>
       <c r="F57" s="1" t="s">
         <v>568</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" ht="197" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>569</v>
       </c>
-      <c r="F58" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="B58" s="1" t="s">
+        <v>577</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>894</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>576</v>
       </c>
+      <c r="B59" t="s">
+        <v>592</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>895</v>
+      </c>
       <c r="F59" s="1" t="s">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>591</v>
       </c>
+      <c r="B60" t="s">
+        <v>606</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>896</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>612</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>282</v>
+      </c>
       <c r="F60" s="1" t="s">
-        <v>603</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="170" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>604</v>
       </c>
+      <c r="B61" s="1" t="s">
+        <v>618</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>620</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>624</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>898</v>
+      </c>
       <c r="F61" s="1" t="s">
-        <v>616</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="187" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>617</v>
       </c>
+      <c r="B62" s="1" t="s">
+        <v>629</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>631</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>624</v>
+      </c>
+      <c r="E62" s="5" t="s">
+        <v>897</v>
+      </c>
       <c r="F62" s="1" t="s">
-        <v>627</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>628</v>
       </c>
+      <c r="B63" s="1" t="s">
+        <v>638</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="F63" s="1" t="s">
-        <v>636</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="340" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>637</v>
       </c>
+      <c r="B64" s="1" t="s">
+        <v>649</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>899</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>900</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="F64" s="1" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="306" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>648</v>
       </c>
+      <c r="B65" s="1" t="s">
+        <v>659</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>901</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>902</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="F65" s="1" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="136" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>658</v>
       </c>
+      <c r="B66" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>904</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="F66" s="1" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="136" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>668</v>
       </c>
+      <c r="B67" s="1" t="s">
+        <v>678</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="F67" s="1" t="s">
-        <v>676</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>677</v>
       </c>
+      <c r="B68" s="1" t="s">
+        <v>685</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>689</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>691</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>146</v>
+      </c>
       <c r="F68" s="1" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>684</v>
       </c>
+      <c r="B69" s="1" t="s">
+        <v>695</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>699</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>702</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>905</v>
+      </c>
       <c r="F69" s="1" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="312" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>694</v>
       </c>
+      <c r="B70" s="1" t="s">
+        <v>709</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>712</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>906</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>716</v>
+      </c>
       <c r="F70" s="1" t="s">
-        <v>707</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="A71" s="1" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="153" x14ac:dyDescent="0.2">
+      <c r="A71" s="6" t="s">
         <v>708</v>
       </c>
+      <c r="B71" t="s">
+        <v>720</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>726</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>61</v>
+      </c>
       <c r="F71" s="1" t="s">
-        <v>718</v>
+        <v>730</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="51" x14ac:dyDescent="0.2">
@@ -10184,103 +10711,100 @@
         <v>719</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>730</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>731</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>740</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>741</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>751</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>761</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>762</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>772</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>773</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>780</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>781</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>792</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>793</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>801</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>802</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>810</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>811</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>821</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>830</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>831</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>839</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>840</v>
-      </c>
-      <c r="F84" s="1" t="s">
-        <v>856</v>
       </c>
     </row>
   </sheetData>

</xml_diff>